<commit_message>
fix: fetch con basePath en todas las páginas client-side
Todas las llamadas fetch('/api/...') ahora usan api('/api/...')
que agrega el prefijo /seguimiento en producción.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cursos.xlsx
+++ b/data/cursos.xlsx
@@ -109,10 +109,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -38720,10 +38719,16 @@
         <v>No</v>
       </c>
       <c r="R699" t="str">
-        <v>En revisión</v>
+        <v>Corrección</v>
       </c>
       <c r="S699" t="str">
         <v>marzo</v>
+      </c>
+      <c r="AB699" t="str">
+        <v>Adela Del Rosario Riveros Flores</v>
+      </c>
+      <c r="AG699" t="str">
+        <v>Corrección</v>
       </c>
     </row>
     <row r="700">
@@ -43225,6 +43230,9 @@
       </c>
       <c r="V836" s="1">
         <v>46156</v>
+      </c>
+      <c r="AB836" t="str">
+        <v>Adela Del Rosario Riveros Flores</v>
       </c>
       <c r="AL836" t="str">
         <v>Calculada</v>
@@ -71567,7 +71575,7 @@
       <c r="Y169" s="1">
         <v>46169.67520408565</v>
       </c>
-      <c r="Z169" s="2">
+      <c r="Z169" s="1">
         <v>46169.675743645836</v>
       </c>
       <c r="AK169" t="str">

</xml_diff>